<commit_message>
adjust jade algo mutation sort
</commit_message>
<xml_diff>
--- a/DE_extension_ExperimentResults.xlsx
+++ b/DE_extension_ExperimentResults.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\MyCode\VisualStudio\meta_algo\DE_extension_to_CEC2005\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F0E4A63-19FD-4EB9-969F-99601C09CCA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6647F26-50C9-41AC-8853-61778255DD37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{50E21A78-8C48-40D2-9105-B406553DA780}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{50E21A78-8C48-40D2-9105-B406553DA780}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
+    <sheet name="工作表2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="36">
   <si>
     <t>f1</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -152,11 +153,43 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>L-SHADE</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>EXPERIMENTAL RESULTS OF 30-DIMENSIONAL PROBLEMS f1– f13, AVERAGED OVER 50 INDEPENDENT RUNS</t>
+    <t>KEY</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Best</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Worst</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">EXPERIMENTAL RESULTS OF </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Microsoft JhengHei Light"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t>30-DIMENSIONAL</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Microsoft JhengHei Light"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t xml:space="preserve"> PROBLEMS f1– f13, AVERAGED OVER 50 INDEPENDENT RUNS</t>
+    </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -167,7 +200,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="0.00000E+00"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -215,6 +248,14 @@
       <family val="2"/>
       <charset val="136"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
+      <name val="Microsoft JhengHei Light"/>
+      <family val="2"/>
+      <charset val="136"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -231,12 +272,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
+        <fgColor theme="7" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -249,8 +290,27 @@
         <color indexed="64"/>
       </left>
       <right/>
-      <top/>
-      <bottom/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -258,16 +318,129 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top/>
-      <bottom/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right/>
-      <top/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -276,80 +449,6 @@
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
       <top style="medium">
         <color indexed="64"/>
       </top>
@@ -364,71 +463,107 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="4" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="4" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="4" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -765,550 +900,994 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44A90AD3-D743-4E65-B2C8-F3B5C98AC2E6}">
-  <dimension ref="B1:K23"/>
+  <dimension ref="B1:K27"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="8.7265625" style="1"/>
     <col min="2" max="2" width="4.08984375" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="48.54296875" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.453125" style="1" customWidth="1"/>
     <col min="6" max="6" width="21" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="21.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.7265625" style="1"/>
+    <col min="8" max="8" width="25.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:11" ht="18.5" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B1" s="17" t="s">
+    <row r="1" spans="2:11" ht="16" thickBot="1" x14ac:dyDescent="0.45"/>
+    <row r="2" spans="2:11" ht="18" x14ac:dyDescent="0.4">
+      <c r="B2" s="31" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="33"/>
+      <c r="J2" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="K2" s="30"/>
+    </row>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.4">
+      <c r="B3" s="7"/>
+      <c r="C3" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="J3" s="14"/>
+      <c r="K3" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-    </row>
-    <row r="2" spans="2:11" x14ac:dyDescent="0.4">
-      <c r="B2" s="7"/>
-      <c r="C2" s="8" t="s">
+    </row>
+    <row r="4" spans="2:11" ht="16" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B4" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2">
+        <v>1500</v>
+      </c>
+      <c r="E4" s="4">
+        <v>4.6552100000000004E-16</v>
+      </c>
+      <c r="F4" s="5">
+        <v>5.1961000000000002E-70</v>
+      </c>
+      <c r="G4" s="5">
+        <v>1.5272100000000001E-66</v>
+      </c>
+      <c r="H4" s="18">
+        <v>2.6419399999999999E-76</v>
+      </c>
+      <c r="J4" s="16"/>
+      <c r="K4" s="17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.4">
+      <c r="B5" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="2">
+        <v>2000</v>
+      </c>
+      <c r="E5" s="4">
+        <v>2.0396199999999999E-13</v>
+      </c>
+      <c r="F5" s="5">
+        <v>3.7009799999999999E-44</v>
+      </c>
+      <c r="G5" s="5">
+        <v>6.2223999999999997E-48</v>
+      </c>
+      <c r="H5" s="18">
+        <v>3.5846600000000003E-52</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" x14ac:dyDescent="0.4">
+      <c r="B6" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="2">
+        <v>5000</v>
+      </c>
+      <c r="E6" s="4">
+        <v>9850.48</v>
+      </c>
+      <c r="F6" s="5">
+        <v>7.9418100000000002E-56</v>
+      </c>
+      <c r="G6" s="6">
+        <v>1.0774399999999999E-86</v>
+      </c>
+      <c r="H6" s="9">
+        <v>1.27133E-79</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.4">
+      <c r="B7" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="2">
+        <v>5000</v>
+      </c>
+      <c r="E7" s="4">
+        <v>5.39516E-7</v>
+      </c>
+      <c r="F7" s="5">
+        <v>4.4286999999999997E-14</v>
+      </c>
+      <c r="G7" s="6">
+        <v>4.5091899999999996E-65</v>
+      </c>
+      <c r="H7" s="9">
+        <v>7.8780800000000003E-52</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" ht="17" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B8" s="23" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="2">
+        <v>3000</v>
+      </c>
+      <c r="E8" s="4">
+        <v>19.126200000000001</v>
+      </c>
+      <c r="F8" s="5">
+        <v>7.9732499999999998E-2</v>
+      </c>
+      <c r="G8" s="5">
+        <v>0.31929999999999997</v>
+      </c>
+      <c r="H8" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.4">
+      <c r="B9" s="23"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="2">
+        <v>20000</v>
+      </c>
+      <c r="E9" s="6">
+        <v>6.5073800000000003E-9</v>
+      </c>
+      <c r="F9" s="5">
+        <v>0.23919699999999999</v>
+      </c>
+      <c r="G9" s="5">
+        <v>7.9732499999999998E-2</v>
+      </c>
+      <c r="H9" s="9">
+        <v>0.159465</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" x14ac:dyDescent="0.4">
+      <c r="B10" s="23" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="2">
+        <v>100</v>
+      </c>
+      <c r="E10" s="4">
+        <v>2998.38</v>
+      </c>
+      <c r="F10" s="6">
+        <v>0.42</v>
+      </c>
+      <c r="G10" s="5">
+        <v>1.6</v>
+      </c>
+      <c r="H10" s="9">
+        <v>2.72</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" x14ac:dyDescent="0.4">
+      <c r="B11" s="23"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="2">
+        <v>1500</v>
+      </c>
+      <c r="E11" s="5">
+        <v>0</v>
+      </c>
+      <c r="F11" s="5">
+        <v>0</v>
+      </c>
+      <c r="G11" s="5">
+        <v>0</v>
+      </c>
+      <c r="H11" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="2:11" x14ac:dyDescent="0.4">
+      <c r="B12" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" s="2">
+        <v>3000</v>
+      </c>
+      <c r="E12" s="5">
+        <v>6.9094200000000003E-3</v>
+      </c>
+      <c r="F12" s="5">
+        <v>6.1007699999999999E-4</v>
+      </c>
+      <c r="G12" s="5">
+        <v>5.1565599999999997E-4</v>
+      </c>
+      <c r="H12" s="9">
+        <v>6.5368200000000005E-4</v>
+      </c>
+    </row>
+    <row r="13" spans="2:11" x14ac:dyDescent="0.4">
+      <c r="B13" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="2">
+        <v>1000</v>
+      </c>
+      <c r="E13" s="4">
+        <v>4664.88</v>
+      </c>
+      <c r="F13" s="5">
+        <v>5.9893299999999997E-2</v>
+      </c>
+      <c r="G13" s="6">
+        <v>2.6538699999999998E-2</v>
+      </c>
+      <c r="H13" s="9">
+        <v>9.6577500000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="2:11" x14ac:dyDescent="0.4">
+      <c r="B14" s="23"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="2">
+        <v>9000</v>
+      </c>
+      <c r="E14" s="4">
+        <v>3439.12</v>
+      </c>
+      <c r="F14" s="6">
+        <v>-3.6379800000000002E-12</v>
+      </c>
+      <c r="G14" s="6">
+        <v>-3.6379800000000002E-12</v>
+      </c>
+      <c r="H14" s="9">
+        <v>4.7375299999999996</v>
+      </c>
+    </row>
+    <row r="15" spans="2:11" x14ac:dyDescent="0.4">
+      <c r="B15" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="D15" s="2">
+        <v>1000</v>
+      </c>
+      <c r="E15" s="4">
+        <v>135.61500000000001</v>
+      </c>
+      <c r="F15" s="5">
+        <v>0.215558</v>
+      </c>
+      <c r="G15" s="5">
+        <v>0.22084500000000001</v>
+      </c>
+      <c r="H15" s="9">
+        <v>3.2317800000000001</v>
+      </c>
+    </row>
+    <row r="16" spans="2:11" x14ac:dyDescent="0.4">
+      <c r="B16" s="23"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="2">
+        <v>5000</v>
+      </c>
+      <c r="E16" s="4">
+        <v>94.655299999999997</v>
+      </c>
+      <c r="F16" s="5">
+        <v>0</v>
+      </c>
+      <c r="G16" s="5">
+        <v>0</v>
+      </c>
+      <c r="H16" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="B17" s="23" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="D17" s="2">
+        <v>500</v>
+      </c>
+      <c r="E17" s="4">
+        <v>3.6448899999999999E-2</v>
+      </c>
+      <c r="F17" s="5">
+        <v>2.51355E-11</v>
+      </c>
+      <c r="G17" s="5">
+        <v>1.0103699999999999E-10</v>
+      </c>
+      <c r="H17" s="9">
+        <v>5.8113E-11</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="B18" s="23"/>
+      <c r="C18" s="22"/>
+      <c r="D18" s="2">
+        <v>2000</v>
+      </c>
+      <c r="E18" s="4">
+        <v>2.5873899999999999E-12</v>
+      </c>
+      <c r="F18" s="5">
+        <v>3.9967999999999998E-15</v>
+      </c>
+      <c r="G18" s="5">
+        <v>3.9967999999999998E-15</v>
+      </c>
+      <c r="H18" s="9">
+        <v>3.9967999999999998E-15</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="B19" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" s="22" t="s">
+        <v>23</v>
+      </c>
+      <c r="D19" s="2">
+        <v>500</v>
+      </c>
+      <c r="E19" s="4">
+        <v>0.10512299999999999</v>
+      </c>
+      <c r="F19" s="5">
+        <v>1.4796899999999999E-4</v>
+      </c>
+      <c r="G19" s="5">
+        <v>1.47995E-4</v>
+      </c>
+      <c r="H19" s="9">
+        <v>1.9714600000000001E-4</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="B20" s="23"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="2">
+        <v>3000</v>
+      </c>
+      <c r="E20" s="5">
+        <v>0</v>
+      </c>
+      <c r="F20" s="5">
+        <v>0</v>
+      </c>
+      <c r="G20" s="5">
+        <v>0</v>
+      </c>
+      <c r="H20" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="B21" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D21" s="2">
+        <v>500</v>
+      </c>
+      <c r="E21" s="4">
+        <v>3.8107500000000002E-2</v>
+      </c>
+      <c r="F21" s="5">
+        <v>1.4300300000000001E-18</v>
+      </c>
+      <c r="G21" s="5">
+        <v>9.72584E-18</v>
+      </c>
+      <c r="H21" s="18">
+        <v>3.1864499999999997E-20</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="B22" s="23"/>
+      <c r="C22" s="22"/>
+      <c r="D22" s="2">
+        <v>1500</v>
+      </c>
+      <c r="E22" s="4">
+        <v>9.9082899999999995E-16</v>
+      </c>
+      <c r="F22" s="5">
+        <v>1.5705400000000001E-32</v>
+      </c>
+      <c r="G22" s="5">
+        <v>1.5705400000000001E-32</v>
+      </c>
+      <c r="H22" s="9">
+        <v>1.5705400000000001E-32</v>
+      </c>
+    </row>
+    <row r="23" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="B23" s="23" t="s">
+        <v>13</v>
+      </c>
+      <c r="C23" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="D23" s="2">
+        <v>500</v>
+      </c>
+      <c r="E23" s="4">
+        <v>9.0445499999999998E-2</v>
+      </c>
+      <c r="F23" s="5">
+        <v>1.8665999999999999E-17</v>
+      </c>
+      <c r="G23" s="5">
+        <v>2.13449E-16</v>
+      </c>
+      <c r="H23" s="18">
+        <v>4.2409199999999998E-19</v>
+      </c>
+    </row>
+    <row r="24" spans="2:8" ht="16" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B24" s="24"/>
+      <c r="C24" s="25"/>
+      <c r="D24" s="10">
+        <v>1500</v>
+      </c>
+      <c r="E24" s="11">
+        <v>2.41746E-15</v>
+      </c>
+      <c r="F24" s="12">
+        <v>1.3497799999999999E-32</v>
+      </c>
+      <c r="G24" s="12">
+        <v>1.3497799999999999E-32</v>
+      </c>
+      <c r="H24" s="13">
+        <v>1.3497799999999999E-32</v>
+      </c>
+    </row>
+    <row r="27" spans="2:8" ht="18" x14ac:dyDescent="0.4">
+      <c r="H27" s="19"/>
+    </row>
+  </sheetData>
+  <mergeCells count="18">
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7242E3B-0CC2-4FB1-9D87-7AA3D39563A7}">
+  <dimension ref="B1:G24"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="2" max="2" width="4.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="50.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.81640625" customWidth="1"/>
+    <col min="6" max="6" width="29" customWidth="1"/>
+    <col min="7" max="7" width="33.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:7" ht="17.5" thickBot="1" x14ac:dyDescent="0.45"/>
+    <row r="2" spans="2:7" ht="18" x14ac:dyDescent="0.4">
+      <c r="B2" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="28"/>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="B3" s="7"/>
+      <c r="C3" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D3" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E3" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F3" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="G3" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="H2" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="I2" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="K2" s="16"/>
-    </row>
-    <row r="3" spans="2:11" x14ac:dyDescent="0.4">
-      <c r="B3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="5" t="s">
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="B4" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="5">
+      <c r="D4" s="2">
         <v>1500</v>
       </c>
-      <c r="E3" s="10">
+      <c r="E4" s="4">
         <v>4.6552100000000004E-16</v>
       </c>
-      <c r="F3" s="12">
+      <c r="F4" s="18">
         <v>5.1961000000000002E-70</v>
       </c>
-      <c r="G3" s="12">
+      <c r="G4" s="9">
         <v>1.5272100000000001E-66</v>
       </c>
-      <c r="H3" s="11">
-        <v>2.6419399999999999E-76</v>
-      </c>
-      <c r="I3" s="3"/>
-    </row>
-    <row r="4" spans="2:11" x14ac:dyDescent="0.4">
-      <c r="B4" s="2" t="s">
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="B5" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D5" s="2">
         <v>2000</v>
       </c>
-      <c r="E4" s="10">
+      <c r="E5" s="4">
         <v>2.0396199999999999E-13</v>
       </c>
-      <c r="F4" s="12">
+      <c r="F5" s="5">
         <v>3.7009799999999999E-44</v>
       </c>
-      <c r="G4" s="12">
+      <c r="G5" s="18">
         <v>6.2223999999999997E-48</v>
       </c>
-      <c r="H4" s="11">
-        <v>3.5846600000000003E-52</v>
-      </c>
-      <c r="I4" s="3"/>
-      <c r="K4" s="15"/>
-    </row>
-    <row r="5" spans="2:11" x14ac:dyDescent="0.4">
-      <c r="B5" s="2" t="s">
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="B6" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D6" s="2">
         <v>5000</v>
       </c>
-      <c r="E5" s="10">
+      <c r="E6" s="4">
         <v>9850.48</v>
       </c>
-      <c r="F5" s="12">
+      <c r="F6" s="5">
         <v>7.9418100000000002E-56</v>
       </c>
-      <c r="G5" s="11">
+      <c r="G6" s="18">
         <v>1.0774399999999999E-86</v>
       </c>
-      <c r="H5" s="12">
-        <v>1.27133E-79</v>
-      </c>
-      <c r="I5" s="3"/>
-    </row>
-    <row r="6" spans="2:11" x14ac:dyDescent="0.4">
-      <c r="B6" s="2" t="s">
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="B7" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D7" s="2">
         <v>5000</v>
       </c>
-      <c r="E6" s="10">
+      <c r="E7" s="4">
         <v>5.39516E-7</v>
       </c>
-      <c r="F6" s="12">
+      <c r="F7" s="5">
         <v>4.4286999999999997E-14</v>
       </c>
-      <c r="G6" s="11">
+      <c r="G7" s="18">
         <v>4.5091899999999996E-65</v>
       </c>
-      <c r="H6" s="12">
-        <v>7.8780800000000003E-52</v>
-      </c>
-      <c r="I6" s="3"/>
-    </row>
-    <row r="7" spans="2:11" ht="17" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B7" s="18" t="s">
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="B8" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="20" t="s">
+      <c r="C8" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D8" s="2">
         <v>3000</v>
       </c>
-      <c r="E7" s="10">
+      <c r="E8" s="4">
         <v>19.126200000000001</v>
       </c>
-      <c r="F7" s="12">
+      <c r="F8" s="5">
         <v>7.9732499999999998E-2</v>
       </c>
-      <c r="G7" s="12">
+      <c r="G8" s="9">
         <v>0.31929999999999997</v>
       </c>
-      <c r="H7" s="11">
-        <v>0</v>
-      </c>
-      <c r="I7" s="3"/>
-    </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.4">
-      <c r="B8" s="18"/>
-      <c r="C8" s="20"/>
-      <c r="D8" s="5">
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="B9" s="23"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="2">
         <v>20000</v>
       </c>
-      <c r="E8" s="11">
+      <c r="E9" s="6">
         <v>6.5073800000000003E-9</v>
       </c>
-      <c r="F8" s="12">
+      <c r="F9" s="5">
         <v>0.23919699999999999</v>
       </c>
-      <c r="G8" s="12">
+      <c r="G9" s="9">
         <v>7.9732499999999998E-2</v>
       </c>
-      <c r="H8" s="12">
-        <v>0.159465</v>
-      </c>
-      <c r="I8" s="3"/>
-    </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.4">
-      <c r="B9" s="18" t="s">
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="B10" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="20" t="s">
+      <c r="C10" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D10" s="2">
         <v>100</v>
       </c>
-      <c r="E9" s="10">
+      <c r="E10" s="4">
         <v>2998.38</v>
       </c>
-      <c r="F9" s="11">
+      <c r="F10" s="6">
         <v>0.42</v>
       </c>
-      <c r="G9" s="12">
+      <c r="G10" s="9">
         <v>1.6</v>
       </c>
-      <c r="H9" s="12">
-        <v>2.72</v>
-      </c>
-      <c r="I9" s="3"/>
-    </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.4">
-      <c r="B10" s="18"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="5">
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="B11" s="23"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="2">
         <v>1500</v>
       </c>
-      <c r="E10" s="12">
-        <v>0</v>
-      </c>
-      <c r="F10" s="12">
-        <v>0</v>
-      </c>
-      <c r="G10" s="12">
-        <v>0</v>
-      </c>
-      <c r="H10" s="12">
-        <v>0</v>
-      </c>
-      <c r="I10" s="3"/>
-    </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.4">
-      <c r="B11" s="2" t="s">
+      <c r="E11" s="5">
+        <v>0</v>
+      </c>
+      <c r="F11" s="5">
+        <v>0</v>
+      </c>
+      <c r="G11" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="B12" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C12" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D12" s="2">
         <v>3000</v>
       </c>
-      <c r="E11" s="12">
+      <c r="E12" s="5">
         <v>6.9094200000000003E-3</v>
       </c>
-      <c r="F11" s="12">
+      <c r="F12" s="5">
         <v>6.1007699999999999E-4</v>
       </c>
-      <c r="G11" s="12">
+      <c r="G12" s="9">
         <v>5.1565599999999997E-4</v>
       </c>
-      <c r="H11" s="12">
-        <v>6.5368200000000005E-4</v>
-      </c>
-      <c r="I11" s="3"/>
-    </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.4">
-      <c r="B12" s="18" t="s">
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="B13" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="20" t="s">
+      <c r="C13" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D13" s="2">
         <v>1000</v>
       </c>
-      <c r="E12" s="10">
+      <c r="E13" s="4">
         <v>4664.88</v>
       </c>
-      <c r="F12" s="12">
+      <c r="F13" s="5">
         <v>5.9893299999999997E-2</v>
       </c>
-      <c r="G12" s="11">
+      <c r="G13" s="18">
         <v>2.6538699999999998E-2</v>
       </c>
-      <c r="H12" s="12">
-        <v>9.6577500000000001</v>
-      </c>
-      <c r="I12" s="3"/>
-    </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.4">
-      <c r="B13" s="18"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="5">
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="B14" s="23"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="2">
         <v>9000</v>
       </c>
-      <c r="E13" s="10">
+      <c r="E14" s="4">
         <v>3439.12</v>
       </c>
-      <c r="F13" s="11">
+      <c r="F14" s="6">
         <v>-3.6379800000000002E-12</v>
       </c>
-      <c r="G13" s="11">
+      <c r="G14" s="18">
         <v>-3.6379800000000002E-12</v>
       </c>
-      <c r="H13" s="12">
-        <v>4.7375299999999996</v>
-      </c>
-      <c r="I13" s="3"/>
-    </row>
-    <row r="14" spans="2:11" x14ac:dyDescent="0.4">
-      <c r="B14" s="18" t="s">
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="B15" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="20" t="s">
+      <c r="C15" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="D14" s="5">
+      <c r="D15" s="2">
         <v>1000</v>
       </c>
-      <c r="E14" s="10">
+      <c r="E15" s="4">
         <v>135.61500000000001</v>
       </c>
-      <c r="F14" s="12">
+      <c r="F15" s="6">
         <v>0.215558</v>
       </c>
-      <c r="G14" s="12">
+      <c r="G15" s="18">
         <v>0.22084500000000001</v>
       </c>
-      <c r="H14" s="12">
-        <v>3.2317800000000001</v>
-      </c>
-      <c r="I14" s="3"/>
-    </row>
-    <row r="15" spans="2:11" x14ac:dyDescent="0.4">
-      <c r="B15" s="18"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="5">
-        <v>5000</v>
-      </c>
-      <c r="E15" s="10">
+    </row>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="B16" s="23"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="2">
+        <v>9000</v>
+      </c>
+      <c r="E16" s="4">
         <v>94.655299999999997</v>
       </c>
-      <c r="F15" s="12">
-        <v>0</v>
-      </c>
-      <c r="G15" s="12">
-        <v>0</v>
-      </c>
-      <c r="H15" s="12">
-        <v>0</v>
-      </c>
-      <c r="I15" s="3"/>
-    </row>
-    <row r="16" spans="2:11" x14ac:dyDescent="0.4">
-      <c r="B16" s="18" t="s">
+      <c r="F16" s="6">
+        <v>0</v>
+      </c>
+      <c r="G16" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="B17" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="C16" s="20" t="s">
+      <c r="C17" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="5">
+      <c r="D17" s="2">
         <v>500</v>
       </c>
-      <c r="E16" s="10">
+      <c r="E17" s="4">
         <v>3.6448899999999999E-2</v>
       </c>
-      <c r="F16" s="12">
+      <c r="F17" s="6">
         <v>2.51355E-11</v>
       </c>
-      <c r="G16" s="12">
+      <c r="G17" s="9">
         <v>1.0103699999999999E-10</v>
       </c>
-      <c r="H16" s="12">
-        <v>5.8113E-11</v>
-      </c>
-      <c r="I16" s="3"/>
-    </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.4">
-      <c r="B17" s="18"/>
-      <c r="C17" s="20"/>
-      <c r="D17" s="5">
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="B18" s="23"/>
+      <c r="C18" s="22"/>
+      <c r="D18" s="2">
         <v>2000</v>
       </c>
-      <c r="E17" s="10">
+      <c r="E18" s="4">
         <v>2.5873899999999999E-12</v>
       </c>
-      <c r="F17" s="12">
+      <c r="F18" s="6">
         <v>3.9967999999999998E-15</v>
       </c>
-      <c r="G17" s="12">
+      <c r="G18" s="18">
         <v>3.9967999999999998E-15</v>
       </c>
-      <c r="H17" s="12">
-        <v>3.9967999999999998E-15</v>
-      </c>
-      <c r="I17" s="3"/>
-    </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.4">
-      <c r="B18" s="18" t="s">
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="B19" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="C18" s="20" t="s">
+      <c r="C19" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="D18" s="5">
+      <c r="D19" s="2">
         <v>500</v>
       </c>
-      <c r="E18" s="10">
+      <c r="E19" s="4">
         <v>0.10512299999999999</v>
       </c>
-      <c r="F18" s="12">
+      <c r="F19" s="6">
         <v>1.4796899999999999E-4</v>
       </c>
-      <c r="G18" s="12">
+      <c r="G19" s="18">
         <v>1.47995E-4</v>
       </c>
-      <c r="H18" s="12">
-        <v>1.9714600000000001E-4</v>
-      </c>
-      <c r="I18" s="3"/>
-    </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.4">
-      <c r="B19" s="18"/>
-      <c r="C19" s="20"/>
-      <c r="D19" s="5">
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="B20" s="23"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="2">
         <v>3000</v>
       </c>
-      <c r="E19" s="12">
-        <v>0</v>
-      </c>
-      <c r="F19" s="12">
-        <v>0</v>
-      </c>
-      <c r="G19" s="12">
-        <v>0</v>
-      </c>
-      <c r="H19" s="12">
-        <v>0</v>
-      </c>
-      <c r="I19" s="3"/>
-    </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.4">
-      <c r="B20" s="18" t="s">
+      <c r="E20" s="5">
+        <v>0</v>
+      </c>
+      <c r="F20" s="5">
+        <v>0</v>
+      </c>
+      <c r="G20" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="B21" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="20" t="s">
+      <c r="C21" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="D20" s="5">
+      <c r="D21" s="2">
         <v>500</v>
       </c>
-      <c r="E20" s="10">
+      <c r="E21" s="4">
         <v>3.8107500000000002E-2</v>
       </c>
-      <c r="F20" s="12">
+      <c r="F21" s="6">
         <v>1.4300300000000001E-18</v>
       </c>
-      <c r="G20" s="12">
+      <c r="G21" s="18">
         <v>9.72584E-18</v>
       </c>
-      <c r="H20" s="11">
-        <v>3.1864499999999997E-20</v>
-      </c>
-      <c r="I20" s="3"/>
-    </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.4">
-      <c r="B21" s="18"/>
-      <c r="C21" s="20"/>
-      <c r="D21" s="5">
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="B22" s="23"/>
+      <c r="C22" s="22"/>
+      <c r="D22" s="2">
         <v>1500</v>
       </c>
-      <c r="E21" s="10">
+      <c r="E22" s="4">
         <v>9.9082899999999995E-16</v>
       </c>
-      <c r="F21" s="12">
+      <c r="F22" s="6">
         <v>1.5705400000000001E-32</v>
       </c>
-      <c r="G21" s="12">
+      <c r="G22" s="18">
         <v>1.5705400000000001E-32</v>
       </c>
-      <c r="H21" s="12">
-        <v>1.5705400000000001E-32</v>
-      </c>
-      <c r="I21" s="3"/>
-    </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.4">
-      <c r="B22" s="18" t="s">
+    </row>
+    <row r="23" spans="2:7" x14ac:dyDescent="0.4">
+      <c r="B23" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="C22" s="20" t="s">
+      <c r="C23" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="D22" s="5">
+      <c r="D23" s="2">
         <v>500</v>
       </c>
-      <c r="E22" s="10">
+      <c r="E23" s="4">
         <v>9.0445499999999998E-2</v>
       </c>
-      <c r="F22" s="12">
+      <c r="F23" s="6">
         <v>1.8665999999999999E-17</v>
       </c>
-      <c r="G22" s="12">
+      <c r="G23" s="9">
         <v>2.13449E-16</v>
       </c>
-      <c r="H22" s="11">
-        <v>4.2409199999999998E-19</v>
-      </c>
-      <c r="I22" s="3"/>
-    </row>
-    <row r="23" spans="2:9" ht="16" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B23" s="19"/>
-      <c r="C23" s="21"/>
-      <c r="D23" s="6">
+    </row>
+    <row r="24" spans="2:7" ht="17.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B24" s="24"/>
+      <c r="C24" s="25"/>
+      <c r="D24" s="10">
         <v>1500</v>
       </c>
-      <c r="E23" s="13">
+      <c r="E24" s="11">
         <v>2.41746E-15</v>
       </c>
-      <c r="F23" s="14">
+      <c r="F24" s="20">
         <v>1.3497799999999999E-32</v>
       </c>
-      <c r="G23" s="14">
+      <c r="G24" s="21">
         <v>1.3497799999999999E-32</v>
       </c>
-      <c r="H23" s="14">
-        <v>1.3497799999999999E-32</v>
-      </c>
-      <c r="I23" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="B1:I1"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>